<commit_message>
correct the mains water temperature model citation from Hendron & Burch (2008) to Burch & Christensen (2007) in ShowerGroundTruthCalculator.py. Reran A_E subset to account for updated examplar, and all architectures have slightly differnet outcome metrics. reran full paper pipeline, updated numbers, upadted paper, and paper refinemnet to be done. also partially cleaned repo.
</commit_message>
<xml_diff>
--- a/Analysis/MetricsSummary/metrics_summary_all_models_imputed_perrun.xlsx
+++ b/Analysis/MetricsSummary/metrics_summary_all_models_imputed_perrun.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.23154</v>
+        <v>0.23142</v>
       </c>
     </row>
     <row r="7">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.3018999999999999</v>
+        <v>0.30174</v>
       </c>
     </row>
     <row r="8">
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.19792</v>
+        <v>0.19736</v>
       </c>
     </row>
     <row r="13">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.32786</v>
+        <v>0.30668</v>
       </c>
     </row>
     <row r="15">
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.35384</v>
+        <v>0.33078</v>
       </c>
     </row>
     <row r="16">
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.5446</v>
+        <v>0.5353800000000001</v>
       </c>
     </row>
     <row r="17">
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.8154</v>
+        <v>0.8112999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -958,7 +958,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.16668</v>
+        <v>0.16772</v>
       </c>
     </row>
     <row r="19">
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.23574</v>
+        <v>0.23652</v>
       </c>
     </row>
     <row r="20">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.41438</v>
+        <v>1.4102</v>
       </c>
     </row>
     <row r="21">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.17478</v>
+        <v>0.17422</v>
       </c>
     </row>
     <row r="23">
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.16438</v>
+        <v>0.16452</v>
       </c>
     </row>
     <row r="24">
@@ -1138,7 +1138,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.17452</v>
+        <v>0.17786</v>
       </c>
     </row>
     <row r="25">
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.15308</v>
+        <v>0.15426</v>
       </c>
     </row>
     <row r="26">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.89734</v>
+        <v>0.89732</v>
       </c>
     </row>
     <row r="27">
@@ -1258,7 +1258,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.90762</v>
+        <v>0.9076000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.04676</v>
+        <v>0.04484</v>
       </c>
     </row>
     <row r="31">
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.09246</v>
+        <v>0.09172</v>
       </c>
     </row>
     <row r="32">
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1.97376</v>
+        <v>2.04072</v>
       </c>
     </row>
     <row r="33">
@@ -1498,7 +1498,7 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0.01672</v>
+        <v>0.008919999999999999</v>
       </c>
     </row>
     <row r="37">
@@ -1678,7 +1678,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>0.21958</v>
+        <v>0.219</v>
       </c>
     </row>
     <row r="43">
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>0.29598</v>
+        <v>0.29534</v>
       </c>
     </row>
     <row r="44">
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1.34796</v>
+        <v>1.34858</v>
       </c>
     </row>
     <row r="45">
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>0.1707</v>
+        <v>0.16834</v>
       </c>
     </row>
     <row r="49">
@@ -1918,7 +1918,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>0.30468</v>
+        <v>0.30986</v>
       </c>
     </row>
     <row r="51">
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>0.32038</v>
+        <v>0.328</v>
       </c>
     </row>
     <row r="52">
@@ -1978,7 +1978,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0.4722000000000001</v>
+        <v>0.48708</v>
       </c>
     </row>
     <row r="53">
@@ -2008,7 +2008,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>0.79366</v>
+        <v>0.79582</v>
       </c>
     </row>
     <row r="54">
@@ -2038,7 +2038,7 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>0.1588</v>
+        <v>0.15838</v>
       </c>
     </row>
     <row r="55">
@@ -2068,7 +2068,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>0.23274</v>
+        <v>0.23114</v>
       </c>
     </row>
     <row r="56">
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>1.46564</v>
+        <v>1.45942</v>
       </c>
     </row>
     <row r="57">
@@ -2128,7 +2128,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="58">
@@ -2158,7 +2158,7 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>0.17822</v>
+        <v>0.17686</v>
       </c>
     </row>
     <row r="59">
@@ -2188,7 +2188,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>0.16668</v>
+        <v>0.16548</v>
       </c>
     </row>
     <row r="60">
@@ -2218,7 +2218,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>0.138</v>
+        <v>0.14004</v>
       </c>
     </row>
     <row r="61">
@@ -2248,7 +2248,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>0.15232</v>
+        <v>0.15112</v>
       </c>
     </row>
     <row r="62">
@@ -2398,7 +2398,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>0.04812</v>
+        <v>0.04768</v>
       </c>
     </row>
     <row r="67">
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>0.1004</v>
+        <v>0.10066</v>
       </c>
     </row>
     <row r="68">
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>2.08652</v>
+        <v>2.11124</v>
       </c>
     </row>
     <row r="69">
@@ -2578,7 +2578,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>0.01082</v>
+        <v>0.00906</v>
       </c>
     </row>
     <row r="73">
@@ -2758,7 +2758,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>0.24152</v>
+        <v>0.24106</v>
       </c>
     </row>
     <row r="79">
@@ -2788,7 +2788,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0.3066</v>
+        <v>0.30628</v>
       </c>
     </row>
     <row r="80">
@@ -2818,7 +2818,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>1.26948</v>
+        <v>1.27058</v>
       </c>
     </row>
     <row r="81">
@@ -2938,7 +2938,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>0.18484</v>
+        <v>0.18314</v>
       </c>
     </row>
     <row r="85">
@@ -2998,7 +2998,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0.27042</v>
+        <v>0.2724799999999999</v>
       </c>
     </row>
     <row r="87">
@@ -3028,7 +3028,7 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>0.28974</v>
+        <v>0.29076</v>
       </c>
     </row>
     <row r="88">
@@ -3058,7 +3058,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0.48</v>
+        <v>0.47386</v>
       </c>
     </row>
     <row r="89">
@@ -3088,7 +3088,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>0.76922</v>
+        <v>0.7651199999999999</v>
       </c>
     </row>
     <row r="90">
@@ -3118,7 +3118,7 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0.16888</v>
+        <v>0.16898</v>
       </c>
     </row>
     <row r="91">
@@ -3148,7 +3148,7 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>0.24304</v>
+        <v>0.24216</v>
       </c>
     </row>
     <row r="92">
@@ -3178,7 +3178,7 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>1.43912</v>
+        <v>1.43308</v>
       </c>
     </row>
     <row r="93">
@@ -3268,7 +3268,7 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>0.1665</v>
+        <v>0.16606</v>
       </c>
     </row>
     <row r="96">
@@ -3298,7 +3298,7 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>0.15362</v>
+        <v>0.155</v>
       </c>
     </row>
     <row r="97">
@@ -3328,7 +3328,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>0.18296</v>
+        <v>0.1824</v>
       </c>
     </row>
     <row r="98">
@@ -3358,7 +3358,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>0.89666</v>
+        <v>0.8974400000000001</v>
       </c>
     </row>
     <row r="99">
@@ -3388,7 +3388,7 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>0.9107799999999999</v>
+        <v>0.9113599999999999</v>
       </c>
     </row>
     <row r="100">
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>0.91616</v>
+        <v>0.9173</v>
       </c>
     </row>
     <row r="101">
@@ -3478,7 +3478,7 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>0.05248000000000001</v>
+        <v>0.05188</v>
       </c>
     </row>
     <row r="103">
@@ -3508,7 +3508,7 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>0.1013</v>
+        <v>0.10148</v>
       </c>
     </row>
     <row r="104">
@@ -3538,7 +3538,7 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>1.92974</v>
+        <v>1.95558</v>
       </c>
     </row>
     <row r="105">
@@ -3658,7 +3658,7 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>0.01266</v>
+        <v>0.01012</v>
       </c>
     </row>
     <row r="109">
@@ -3838,7 +3838,7 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>0.23496</v>
+        <v>0.23486</v>
       </c>
     </row>
     <row r="115">
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="F115" t="n">
-        <v>0.29522</v>
+        <v>0.2948</v>
       </c>
     </row>
     <row r="116">
@@ -3898,7 +3898,7 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1.25648</v>
+        <v>1.25524</v>
       </c>
     </row>
     <row r="117">
@@ -4018,7 +4018,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>0.19472</v>
+        <v>0.19428</v>
       </c>
     </row>
     <row r="121">
@@ -4078,7 +4078,7 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>0.20684</v>
+        <v>0.2082</v>
       </c>
     </row>
     <row r="123">
@@ -4108,7 +4108,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>0.22204</v>
+        <v>0.22412</v>
       </c>
     </row>
     <row r="124">
@@ -4138,7 +4138,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>0.46976</v>
+        <v>0.46566</v>
       </c>
     </row>
     <row r="125">
@@ -4168,7 +4168,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>0.7682</v>
+        <v>0.7805199999999999</v>
       </c>
     </row>
     <row r="126">
@@ -4198,7 +4198,7 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>0.19132</v>
+        <v>0.19354</v>
       </c>
     </row>
     <row r="127">
@@ -4228,7 +4228,7 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>0.2588</v>
+        <v>0.26056</v>
       </c>
     </row>
     <row r="128">
@@ -4258,7 +4258,7 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>1.35274</v>
+        <v>1.3463</v>
       </c>
     </row>
     <row r="129">
@@ -4318,7 +4318,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>0.19502</v>
+        <v>0.19752</v>
       </c>
     </row>
     <row r="131">
@@ -4348,7 +4348,7 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>0.19186</v>
+        <v>0.19466</v>
       </c>
     </row>
     <row r="132">
@@ -4378,7 +4378,7 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>0.19272</v>
+        <v>0.19306</v>
       </c>
     </row>
     <row r="133">
@@ -4408,7 +4408,7 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>0.18576</v>
+        <v>0.18888</v>
       </c>
     </row>
     <row r="134">
@@ -4558,7 +4558,7 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>0.07221999999999999</v>
+        <v>0.07178</v>
       </c>
     </row>
     <row r="139">
@@ -4588,7 +4588,7 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>0.16192</v>
+        <v>0.16208</v>
       </c>
     </row>
     <row r="140">
@@ -4618,7 +4618,7 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>2.24196</v>
+        <v>2.25796</v>
       </c>
     </row>
     <row r="141">
@@ -4738,7 +4738,7 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>0.01076</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="145">
@@ -4918,7 +4918,7 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>0.23184</v>
+        <v>0.23172</v>
       </c>
     </row>
     <row r="151">
@@ -4948,7 +4948,7 @@
         </is>
       </c>
       <c r="F151" t="n">
-        <v>0.30208</v>
+        <v>0.30194</v>
       </c>
     </row>
     <row r="152">
@@ -4978,7 +4978,7 @@
         </is>
       </c>
       <c r="F152" t="n">
-        <v>1.30302</v>
+        <v>1.30306</v>
       </c>
     </row>
     <row r="153">
@@ -5098,7 +5098,7 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>0.19866</v>
+        <v>0.19818</v>
       </c>
     </row>
     <row r="157">
@@ -5158,7 +5158,7 @@
         </is>
       </c>
       <c r="F158" t="n">
-        <v>0.32786</v>
+        <v>0.30668</v>
       </c>
     </row>
     <row r="159">
@@ -5188,7 +5188,7 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>0.35384</v>
+        <v>0.33078</v>
       </c>
     </row>
     <row r="160">
@@ -5218,7 +5218,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>0.5446</v>
+        <v>0.5353800000000001</v>
       </c>
     </row>
     <row r="161">
@@ -5248,7 +5248,7 @@
         </is>
       </c>
       <c r="F161" t="n">
-        <v>0.8154</v>
+        <v>0.8112999999999999</v>
       </c>
     </row>
     <row r="162">
@@ -5278,7 +5278,7 @@
         </is>
       </c>
       <c r="F162" t="n">
-        <v>0.16668</v>
+        <v>0.16772</v>
       </c>
     </row>
     <row r="163">
@@ -5308,7 +5308,7 @@
         </is>
       </c>
       <c r="F163" t="n">
-        <v>0.23574</v>
+        <v>0.23652</v>
       </c>
     </row>
     <row r="164">
@@ -5338,7 +5338,7 @@
         </is>
       </c>
       <c r="F164" t="n">
-        <v>1.41438</v>
+        <v>1.4102</v>
       </c>
     </row>
     <row r="165">
@@ -5398,7 +5398,7 @@
         </is>
       </c>
       <c r="F166" t="n">
-        <v>0.17478</v>
+        <v>0.17422</v>
       </c>
     </row>
     <row r="167">
@@ -5428,7 +5428,7 @@
         </is>
       </c>
       <c r="F167" t="n">
-        <v>0.16438</v>
+        <v>0.16452</v>
       </c>
     </row>
     <row r="168">
@@ -5458,7 +5458,7 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>0.17452</v>
+        <v>0.17786</v>
       </c>
     </row>
     <row r="169">
@@ -5488,7 +5488,7 @@
         </is>
       </c>
       <c r="F169" t="n">
-        <v>0.15308</v>
+        <v>0.15426</v>
       </c>
     </row>
     <row r="170">
@@ -5548,7 +5548,7 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>0.9097199999999999</v>
+        <v>0.90974</v>
       </c>
     </row>
     <row r="172">
@@ -5578,7 +5578,7 @@
         </is>
       </c>
       <c r="F172" t="n">
-        <v>0.9066799999999999</v>
+        <v>0.90668</v>
       </c>
     </row>
     <row r="173">
@@ -5638,7 +5638,7 @@
         </is>
       </c>
       <c r="F174" t="n">
-        <v>0.04681999999999999</v>
+        <v>0.04492</v>
       </c>
     </row>
     <row r="175">
@@ -5668,7 +5668,7 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>0.09258000000000001</v>
+        <v>0.09184</v>
       </c>
     </row>
     <row r="176">
@@ -5698,7 +5698,7 @@
         </is>
       </c>
       <c r="F176" t="n">
-        <v>1.97376</v>
+        <v>2.03976</v>
       </c>
     </row>
     <row r="177">
@@ -5818,7 +5818,7 @@
         </is>
       </c>
       <c r="F180" t="n">
-        <v>0.01704</v>
+        <v>0.00924</v>
       </c>
     </row>
     <row r="181">
@@ -5998,7 +5998,7 @@
         </is>
       </c>
       <c r="F186" t="n">
-        <v>0.21958</v>
+        <v>0.219</v>
       </c>
     </row>
     <row r="187">
@@ -6028,7 +6028,7 @@
         </is>
       </c>
       <c r="F187" t="n">
-        <v>0.29598</v>
+        <v>0.29534</v>
       </c>
     </row>
     <row r="188">
@@ -6058,7 +6058,7 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>1.34796</v>
+        <v>1.34858</v>
       </c>
     </row>
     <row r="189">
@@ -6178,7 +6178,7 @@
         </is>
       </c>
       <c r="F192" t="n">
-        <v>0.1707</v>
+        <v>0.16834</v>
       </c>
     </row>
     <row r="193">
@@ -6238,7 +6238,7 @@
         </is>
       </c>
       <c r="F194" t="n">
-        <v>0.31008</v>
+        <v>0.30872</v>
       </c>
     </row>
     <row r="195">
@@ -6268,7 +6268,7 @@
         </is>
       </c>
       <c r="F195" t="n">
-        <v>0.32566</v>
+        <v>0.3266600000000001</v>
       </c>
     </row>
     <row r="196">
@@ -6298,7 +6298,7 @@
         </is>
       </c>
       <c r="F196" t="n">
-        <v>0.47794</v>
+        <v>0.48822</v>
       </c>
     </row>
     <row r="197">
@@ -6358,7 +6358,7 @@
         </is>
       </c>
       <c r="F198" t="n">
-        <v>0.161</v>
+        <v>0.15992</v>
       </c>
     </row>
     <row r="199">
@@ -6388,7 +6388,7 @@
         </is>
       </c>
       <c r="F199" t="n">
-        <v>0.23462</v>
+        <v>0.23264</v>
       </c>
     </row>
     <row r="200">
@@ -6418,7 +6418,7 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>1.45736</v>
+        <v>1.45472</v>
       </c>
     </row>
     <row r="201">
@@ -6478,7 +6478,7 @@
         </is>
       </c>
       <c r="F202" t="n">
-        <v>0.1805</v>
+        <v>0.17882</v>
       </c>
     </row>
     <row r="203">
@@ -6508,7 +6508,7 @@
         </is>
       </c>
       <c r="F203" t="n">
-        <v>0.16932</v>
+        <v>0.16762</v>
       </c>
     </row>
     <row r="204">
@@ -6538,7 +6538,7 @@
         </is>
       </c>
       <c r="F204" t="n">
-        <v>0.14114</v>
+        <v>0.1413</v>
       </c>
     </row>
     <row r="205">
@@ -6568,7 +6568,7 @@
         </is>
       </c>
       <c r="F205" t="n">
-        <v>0.15314</v>
+        <v>0.15198</v>
       </c>
     </row>
     <row r="206">
@@ -6718,7 +6718,7 @@
         </is>
       </c>
       <c r="F210" t="n">
-        <v>0.04812</v>
+        <v>0.04768</v>
       </c>
     </row>
     <row r="211">
@@ -6748,7 +6748,7 @@
         </is>
       </c>
       <c r="F211" t="n">
-        <v>0.1004</v>
+        <v>0.10066</v>
       </c>
     </row>
     <row r="212">
@@ -6778,7 +6778,7 @@
         </is>
       </c>
       <c r="F212" t="n">
-        <v>2.08652</v>
+        <v>2.11124</v>
       </c>
     </row>
     <row r="213">
@@ -6898,7 +6898,7 @@
         </is>
       </c>
       <c r="F216" t="n">
-        <v>0.01082</v>
+        <v>0.00906</v>
       </c>
     </row>
     <row r="217">
@@ -7078,7 +7078,7 @@
         </is>
       </c>
       <c r="F222" t="n">
-        <v>0.24152</v>
+        <v>0.24106</v>
       </c>
     </row>
     <row r="223">
@@ -7108,7 +7108,7 @@
         </is>
       </c>
       <c r="F223" t="n">
-        <v>0.3066</v>
+        <v>0.30628</v>
       </c>
     </row>
     <row r="224">
@@ -7138,7 +7138,7 @@
         </is>
       </c>
       <c r="F224" t="n">
-        <v>1.26948</v>
+        <v>1.27058</v>
       </c>
     </row>
     <row r="225">
@@ -7258,7 +7258,7 @@
         </is>
       </c>
       <c r="F228" t="n">
-        <v>0.18484</v>
+        <v>0.18314</v>
       </c>
     </row>
     <row r="229">
@@ -7318,7 +7318,7 @@
         </is>
       </c>
       <c r="F230" t="n">
-        <v>0.27042</v>
+        <v>0.2724799999999999</v>
       </c>
     </row>
     <row r="231">
@@ -7348,7 +7348,7 @@
         </is>
       </c>
       <c r="F231" t="n">
-        <v>0.28974</v>
+        <v>0.29076</v>
       </c>
     </row>
     <row r="232">
@@ -7378,7 +7378,7 @@
         </is>
       </c>
       <c r="F232" t="n">
-        <v>0.48</v>
+        <v>0.47386</v>
       </c>
     </row>
     <row r="233">
@@ -7408,7 +7408,7 @@
         </is>
       </c>
       <c r="F233" t="n">
-        <v>0.76922</v>
+        <v>0.7651199999999999</v>
       </c>
     </row>
     <row r="234">
@@ -7438,7 +7438,7 @@
         </is>
       </c>
       <c r="F234" t="n">
-        <v>0.16888</v>
+        <v>0.16898</v>
       </c>
     </row>
     <row r="235">
@@ -7468,7 +7468,7 @@
         </is>
       </c>
       <c r="F235" t="n">
-        <v>0.24304</v>
+        <v>0.24216</v>
       </c>
     </row>
     <row r="236">
@@ -7498,7 +7498,7 @@
         </is>
       </c>
       <c r="F236" t="n">
-        <v>1.43912</v>
+        <v>1.43308</v>
       </c>
     </row>
     <row r="237">
@@ -7588,7 +7588,7 @@
         </is>
       </c>
       <c r="F239" t="n">
-        <v>0.1665</v>
+        <v>0.16606</v>
       </c>
     </row>
     <row r="240">
@@ -7618,7 +7618,7 @@
         </is>
       </c>
       <c r="F240" t="n">
-        <v>0.15362</v>
+        <v>0.155</v>
       </c>
     </row>
     <row r="241">
@@ -7648,7 +7648,7 @@
         </is>
       </c>
       <c r="F241" t="n">
-        <v>0.18296</v>
+        <v>0.1824</v>
       </c>
     </row>
     <row r="242">
@@ -7678,7 +7678,7 @@
         </is>
       </c>
       <c r="F242" t="n">
-        <v>0.78598</v>
+        <v>0.78666</v>
       </c>
     </row>
     <row r="243">
@@ -7708,7 +7708,7 @@
         </is>
       </c>
       <c r="F243" t="n">
-        <v>0.79794</v>
+        <v>0.7984600000000001</v>
       </c>
     </row>
     <row r="244">
@@ -7738,7 +7738,7 @@
         </is>
       </c>
       <c r="F244" t="n">
-        <v>0.8359</v>
+        <v>0.83694</v>
       </c>
     </row>
     <row r="245">
@@ -7798,7 +7798,7 @@
         </is>
       </c>
       <c r="F246" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.07716000000000001</v>
       </c>
     </row>
     <row r="247">
@@ -7828,7 +7828,7 @@
         </is>
       </c>
       <c r="F247" t="n">
-        <v>0.14052</v>
+        <v>0.14066</v>
       </c>
     </row>
     <row r="248">
@@ -7858,7 +7858,7 @@
         </is>
       </c>
       <c r="F248" t="n">
-        <v>1.80876</v>
+        <v>1.82332</v>
       </c>
     </row>
     <row r="249">
@@ -7978,7 +7978,7 @@
         </is>
       </c>
       <c r="F252" t="n">
-        <v>0.04404</v>
+        <v>0.04178</v>
       </c>
     </row>
     <row r="253">
@@ -8158,7 +8158,7 @@
         </is>
       </c>
       <c r="F258" t="n">
-        <v>0.23502</v>
+        <v>0.23492</v>
       </c>
     </row>
     <row r="259">
@@ -8188,7 +8188,7 @@
         </is>
       </c>
       <c r="F259" t="n">
-        <v>0.29526</v>
+        <v>0.29484</v>
       </c>
     </row>
     <row r="260">
@@ -8218,7 +8218,7 @@
         </is>
       </c>
       <c r="F260" t="n">
-        <v>1.25634</v>
+        <v>1.25508</v>
       </c>
     </row>
     <row r="261">
@@ -8338,7 +8338,7 @@
         </is>
       </c>
       <c r="F264" t="n">
-        <v>0.19482</v>
+        <v>0.1944</v>
       </c>
     </row>
     <row r="265">
@@ -8398,7 +8398,7 @@
         </is>
       </c>
       <c r="F266" t="n">
-        <v>0.20684</v>
+        <v>0.2082</v>
       </c>
     </row>
     <row r="267">
@@ -8428,7 +8428,7 @@
         </is>
       </c>
       <c r="F267" t="n">
-        <v>0.22204</v>
+        <v>0.22412</v>
       </c>
     </row>
     <row r="268">
@@ -8458,7 +8458,7 @@
         </is>
       </c>
       <c r="F268" t="n">
-        <v>0.46976</v>
+        <v>0.46566</v>
       </c>
     </row>
     <row r="269">
@@ -8488,7 +8488,7 @@
         </is>
       </c>
       <c r="F269" t="n">
-        <v>0.7682</v>
+        <v>0.7805199999999999</v>
       </c>
     </row>
     <row r="270">
@@ -8518,7 +8518,7 @@
         </is>
       </c>
       <c r="F270" t="n">
-        <v>0.19132</v>
+        <v>0.19354</v>
       </c>
     </row>
     <row r="271">
@@ -8548,7 +8548,7 @@
         </is>
       </c>
       <c r="F271" t="n">
-        <v>0.2588</v>
+        <v>0.26056</v>
       </c>
     </row>
     <row r="272">
@@ -8578,7 +8578,7 @@
         </is>
       </c>
       <c r="F272" t="n">
-        <v>1.35274</v>
+        <v>1.3463</v>
       </c>
     </row>
     <row r="273">
@@ -8638,7 +8638,7 @@
         </is>
       </c>
       <c r="F274" t="n">
-        <v>0.19502</v>
+        <v>0.19752</v>
       </c>
     </row>
     <row r="275">
@@ -8668,7 +8668,7 @@
         </is>
       </c>
       <c r="F275" t="n">
-        <v>0.19186</v>
+        <v>0.19466</v>
       </c>
     </row>
     <row r="276">
@@ -8698,7 +8698,7 @@
         </is>
       </c>
       <c r="F276" t="n">
-        <v>0.19272</v>
+        <v>0.19306</v>
       </c>
     </row>
     <row r="277">
@@ -8728,7 +8728,7 @@
         </is>
       </c>
       <c r="F277" t="n">
-        <v>0.18576</v>
+        <v>0.18888</v>
       </c>
     </row>
     <row r="278">
@@ -8878,7 +8878,7 @@
         </is>
       </c>
       <c r="F282" t="n">
-        <v>0.07256</v>
+        <v>0.07211999999999999</v>
       </c>
     </row>
     <row r="283">
@@ -8908,7 +8908,7 @@
         </is>
       </c>
       <c r="F283" t="n">
-        <v>0.16224</v>
+        <v>0.16238</v>
       </c>
     </row>
     <row r="284">
@@ -8938,7 +8938,7 @@
         </is>
       </c>
       <c r="F284" t="n">
-        <v>2.23592</v>
+        <v>2.25152</v>
       </c>
     </row>
     <row r="285">
@@ -9058,7 +9058,7 @@
         </is>
       </c>
       <c r="F288" t="n">
-        <v>0.0113</v>
+        <v>0.00954</v>
       </c>
     </row>
     <row r="289">
@@ -9165,13 +9165,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.2319000000000001</v>
+        <v>0.231585</v>
       </c>
       <c r="D3" t="n">
-        <v>0.23199</v>
+        <v>0.231675</v>
       </c>
       <c r="E3" t="n">
-        <v>8.999999999997899e-05</v>
+        <v>9.000000000000674e-05</v>
       </c>
     </row>
     <row r="4">
@@ -9207,13 +9207,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.27745</v>
+        <v>0.274305</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2788</v>
+        <v>0.27402</v>
       </c>
       <c r="E5" t="n">
-        <v>0.001350000000000018</v>
+        <v>-0.0002849999999999797</v>
       </c>
     </row>
     <row r="6">
@@ -9228,13 +9228,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.17142</v>
+        <v>0.172155</v>
       </c>
       <c r="D6" t="n">
-        <v>0.17197</v>
+        <v>0.17254</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0005499999999999949</v>
+        <v>0.0003850000000000242</v>
       </c>
     </row>
     <row r="7">
@@ -9249,13 +9249,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.49164</v>
+        <v>0.490495</v>
       </c>
       <c r="D7" t="n">
-        <v>0.493075</v>
+        <v>0.49078</v>
       </c>
       <c r="E7" t="n">
-        <v>0.00143500000000002</v>
+        <v>0.0002849999999999797</v>
       </c>
     </row>
     <row r="8">
@@ -9270,13 +9270,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.899385</v>
+        <v>0.899575</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8707750000000001</v>
+        <v>0.8709450000000001</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.02860999999999991</v>
+        <v>-0.02862999999999993</v>
       </c>
     </row>
     <row r="9">
@@ -9291,13 +9291,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.054895</v>
+        <v>0.054045</v>
       </c>
       <c r="D9" t="n">
-        <v>0.06130000000000001</v>
+        <v>0.06047</v>
       </c>
       <c r="E9" t="n">
-        <v>0.006405000000000008</v>
+        <v>0.006425000000000007</v>
       </c>
     </row>
     <row r="10">
@@ -9312,13 +9312,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.91307</v>
+        <v>0.91335</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8923049999999999</v>
+        <v>0.8925649999999999</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.02076500000000014</v>
+        <v>-0.02078500000000005</v>
       </c>
     </row>
   </sheetData>
@@ -9543,22 +9543,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H6" t="n">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="I6" t="n">
         <v>195</v>
@@ -9955,10 +9955,10 @@
         <v>0.7538</v>
       </c>
       <c r="N2" t="n">
-        <v>0.233</v>
+        <v>0.2328</v>
       </c>
       <c r="O2" t="n">
-        <v>0.3025</v>
+        <v>0.3024</v>
       </c>
     </row>
     <row r="3">
@@ -10006,7 +10006,7 @@
         <v>0.7282</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2291</v>
+        <v>0.2293</v>
       </c>
       <c r="O3" t="n">
         <v>0.3006</v>
@@ -10060,7 +10060,7 @@
         <v>0.2363</v>
       </c>
       <c r="O4" t="n">
-        <v>0.3076</v>
+        <v>0.3075</v>
       </c>
     </row>
     <row r="5">
@@ -10108,10 +10108,10 @@
         <v>0.7128</v>
       </c>
       <c r="N5" t="n">
-        <v>0.2312</v>
+        <v>0.231</v>
       </c>
       <c r="O5" t="n">
-        <v>0.2987</v>
+        <v>0.2986</v>
       </c>
     </row>
     <row r="6">
@@ -10159,10 +10159,10 @@
         <v>0.7128</v>
       </c>
       <c r="N6" t="n">
-        <v>0.2296</v>
+        <v>0.2292</v>
       </c>
       <c r="O6" t="n">
-        <v>0.301</v>
+        <v>0.3006</v>
       </c>
     </row>
     <row r="7">
@@ -10198,19 +10198,19 @@
         <v>195</v>
       </c>
       <c r="J7" t="n">
-        <v>0.3299</v>
+        <v>0.3436</v>
       </c>
       <c r="K7" t="n">
-        <v>0.3564</v>
+        <v>0.3615</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5692</v>
+        <v>0.5744</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7949000000000001</v>
+        <v>0.8051</v>
       </c>
       <c r="N7" t="n">
-        <v>0.1675</v>
+        <v>0.1682</v>
       </c>
       <c r="O7" t="n">
         <v>0.2376</v>
@@ -10249,22 +10249,22 @@
         <v>195</v>
       </c>
       <c r="J8" t="n">
-        <v>0.3162</v>
+        <v>0.3368</v>
       </c>
       <c r="K8" t="n">
-        <v>0.3462</v>
+        <v>0.3667</v>
       </c>
       <c r="L8" t="n">
-        <v>0.5436</v>
+        <v>0.5641</v>
       </c>
       <c r="M8" t="n">
-        <v>0.8359</v>
+        <v>0.8462</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1655</v>
+        <v>0.1667</v>
       </c>
       <c r="O8" t="n">
-        <v>0.2347</v>
+        <v>0.2346</v>
       </c>
     </row>
     <row r="9">
@@ -10300,22 +10300,22 @@
         <v>195</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2855</v>
+        <v>0.2581</v>
       </c>
       <c r="K9" t="n">
-        <v>0.3128</v>
+        <v>0.2821</v>
       </c>
       <c r="L9" t="n">
-        <v>0.5077</v>
+        <v>0.4974</v>
       </c>
       <c r="M9" t="n">
         <v>0.8103</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1675</v>
+        <v>0.168</v>
       </c>
       <c r="O9" t="n">
-        <v>0.2364</v>
+        <v>0.2366</v>
       </c>
     </row>
     <row r="10">
@@ -10351,22 +10351,22 @@
         <v>195</v>
       </c>
       <c r="J10" t="n">
-        <v>0.3573</v>
+        <v>0.2855</v>
       </c>
       <c r="K10" t="n">
-        <v>0.3769</v>
+        <v>0.3026</v>
       </c>
       <c r="L10" t="n">
-        <v>0.5487</v>
+        <v>0.5282</v>
       </c>
       <c r="M10" t="n">
-        <v>0.8154</v>
+        <v>0.7795</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1638</v>
+        <v>0.1674</v>
       </c>
       <c r="O10" t="n">
-        <v>0.233</v>
+        <v>0.2374</v>
       </c>
     </row>
     <row r="11">
@@ -10402,22 +10402,22 @@
         <v>195</v>
       </c>
       <c r="J11" t="n">
-        <v>0.3504</v>
+        <v>0.3094</v>
       </c>
       <c r="K11" t="n">
-        <v>0.3769</v>
+        <v>0.341</v>
       </c>
       <c r="L11" t="n">
-        <v>0.5538</v>
+        <v>0.5128</v>
       </c>
       <c r="M11" t="n">
-        <v>0.8205</v>
+        <v>0.8154</v>
       </c>
       <c r="N11" t="n">
-        <v>0.1691</v>
+        <v>0.1683</v>
       </c>
       <c r="O11" t="n">
-        <v>0.237</v>
+        <v>0.2364</v>
       </c>
     </row>
     <row r="12">
@@ -10465,10 +10465,10 @@
         <v>0.9846</v>
       </c>
       <c r="N12" t="n">
-        <v>0.0399</v>
+        <v>0.0395</v>
       </c>
       <c r="O12" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.0781</v>
       </c>
     </row>
     <row r="13">
@@ -10504,22 +10504,22 @@
         <v>195</v>
       </c>
       <c r="J13" t="n">
-        <v>0.8905999999999999</v>
+        <v>0.8872</v>
       </c>
       <c r="K13" t="n">
-        <v>0.9051</v>
+        <v>0.9026</v>
       </c>
       <c r="L13" t="n">
-        <v>0.8974</v>
+        <v>0.8923</v>
       </c>
       <c r="M13" t="n">
         <v>0.9744</v>
       </c>
       <c r="N13" t="n">
-        <v>0.0487</v>
+        <v>0.0469</v>
       </c>
       <c r="O13" t="n">
-        <v>0.0969</v>
+        <v>0.0963</v>
       </c>
     </row>
     <row r="14">
@@ -10567,10 +10567,10 @@
         <v>0.9744</v>
       </c>
       <c r="N14" t="n">
-        <v>0.0486</v>
+        <v>0.0462</v>
       </c>
       <c r="O14" t="n">
-        <v>0.0954</v>
+        <v>0.09429999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -10618,10 +10618,10 @@
         <v>0.9795</v>
       </c>
       <c r="N15" t="n">
-        <v>0.0452</v>
+        <v>0.0427</v>
       </c>
       <c r="O15" t="n">
-        <v>0.0854</v>
+        <v>0.0839</v>
       </c>
     </row>
     <row r="16">
@@ -10657,22 +10657,22 @@
         <v>195</v>
       </c>
       <c r="J16" t="n">
-        <v>0.894</v>
+        <v>0.8974</v>
       </c>
       <c r="K16" t="n">
+        <v>0.9103</v>
+      </c>
+      <c r="L16" t="n">
         <v>0.9077</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0.9026</v>
       </c>
       <c r="M16" t="n">
         <v>0.9744</v>
       </c>
       <c r="N16" t="n">
-        <v>0.0517</v>
+        <v>0.0493</v>
       </c>
       <c r="O16" t="n">
-        <v>0.1075</v>
+        <v>0.1066</v>
       </c>
     </row>
     <row r="17">
@@ -10720,10 +10720,10 @@
         <v>0.7026</v>
       </c>
       <c r="N17" t="n">
-        <v>0.2171</v>
+        <v>0.2164</v>
       </c>
       <c r="O17" t="n">
-        <v>0.2929</v>
+        <v>0.2922</v>
       </c>
     </row>
     <row r="18">
@@ -10771,10 +10771,10 @@
         <v>0.6718</v>
       </c>
       <c r="N18" t="n">
-        <v>0.2193</v>
+        <v>0.2188</v>
       </c>
       <c r="O18" t="n">
-        <v>0.2966</v>
+        <v>0.296</v>
       </c>
     </row>
     <row r="19">
@@ -10822,10 +10822,10 @@
         <v>0.7077</v>
       </c>
       <c r="N19" t="n">
-        <v>0.2203</v>
+        <v>0.2198</v>
       </c>
       <c r="O19" t="n">
-        <v>0.2968</v>
+        <v>0.2961</v>
       </c>
     </row>
     <row r="20">
@@ -10873,10 +10873,10 @@
         <v>0.6923</v>
       </c>
       <c r="N20" t="n">
-        <v>0.2215</v>
+        <v>0.2209</v>
       </c>
       <c r="O20" t="n">
-        <v>0.2976</v>
+        <v>0.297</v>
       </c>
     </row>
     <row r="21">
@@ -10924,10 +10924,10 @@
         <v>0.7128</v>
       </c>
       <c r="N21" t="n">
-        <v>0.2197</v>
+        <v>0.2191</v>
       </c>
       <c r="O21" t="n">
-        <v>0.296</v>
+        <v>0.2954</v>
       </c>
     </row>
     <row r="22">
@@ -10953,10 +10953,10 @@
         <v>195</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
@@ -10966,19 +10966,19 @@
         <v>0.2786</v>
       </c>
       <c r="K22" t="n">
-        <v>0.2949</v>
+        <v>0.2974</v>
       </c>
       <c r="L22" t="n">
-        <v>0.4564</v>
+        <v>0.4667</v>
       </c>
       <c r="M22" t="n">
         <v>0.8</v>
       </c>
       <c r="N22" t="n">
-        <v>0.1596</v>
+        <v>0.1591</v>
       </c>
       <c r="O22" t="n">
-        <v>0.2342</v>
+        <v>0.2328</v>
       </c>
     </row>
     <row r="23">
@@ -11014,22 +11014,22 @@
         <v>195</v>
       </c>
       <c r="J23" t="n">
-        <v>0.3333</v>
+        <v>0.3299</v>
       </c>
       <c r="K23" t="n">
         <v>0.3513</v>
       </c>
       <c r="L23" t="n">
-        <v>0.5077</v>
+        <v>0.5128</v>
       </c>
       <c r="M23" t="n">
         <v>0.7949000000000001</v>
       </c>
       <c r="N23" t="n">
-        <v>0.1596</v>
+        <v>0.1598</v>
       </c>
       <c r="O23" t="n">
-        <v>0.2337</v>
+        <v>0.233</v>
       </c>
     </row>
     <row r="24">
@@ -11055,32 +11055,32 @@
         <v>195</v>
       </c>
       <c r="F24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G24" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
         <v>195</v>
       </c>
       <c r="J24" t="n">
-        <v>0.306</v>
+        <v>0.2923</v>
       </c>
       <c r="K24" t="n">
-        <v>0.3231</v>
+        <v>0.3128</v>
       </c>
       <c r="L24" t="n">
-        <v>0.4769</v>
+        <v>0.4667</v>
       </c>
       <c r="M24" t="n">
         <v>0.7897</v>
       </c>
       <c r="N24" t="n">
-        <v>0.1604</v>
+        <v>0.1603</v>
       </c>
       <c r="O24" t="n">
-        <v>0.2343</v>
+        <v>0.2331</v>
       </c>
     </row>
     <row r="25">
@@ -11106,32 +11106,32 @@
         <v>195</v>
       </c>
       <c r="F25" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G25" t="n">
-        <v>84</v>
+        <v>24</v>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
         <v>195</v>
       </c>
       <c r="J25" t="n">
-        <v>0.3197</v>
+        <v>0.3231</v>
       </c>
       <c r="K25" t="n">
-        <v>0.3308</v>
+        <v>0.3359</v>
       </c>
       <c r="L25" t="n">
-        <v>0.4769</v>
+        <v>0.4923</v>
       </c>
       <c r="M25" t="n">
         <v>0.7949000000000001</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1638</v>
+        <v>0.1591</v>
       </c>
       <c r="O25" t="n">
-        <v>0.2358</v>
+        <v>0.2307</v>
       </c>
     </row>
     <row r="26">
@@ -11157,32 +11157,32 @@
         <v>195</v>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G26" t="n">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
         <v>195</v>
       </c>
       <c r="J26" t="n">
-        <v>0.3128</v>
+        <v>0.3197</v>
       </c>
       <c r="K26" t="n">
-        <v>0.3282</v>
+        <v>0.3359</v>
       </c>
       <c r="L26" t="n">
-        <v>0.4718</v>
+        <v>0.5026</v>
       </c>
       <c r="M26" t="n">
         <v>0.8</v>
       </c>
       <c r="N26" t="n">
-        <v>0.1616</v>
+        <v>0.1613</v>
       </c>
       <c r="O26" t="n">
-        <v>0.2351</v>
+        <v>0.2336</v>
       </c>
     </row>
     <row r="27">
@@ -11230,10 +11230,10 @@
         <v>0.9846</v>
       </c>
       <c r="N27" t="n">
-        <v>0.0474</v>
+        <v>0.0469</v>
       </c>
       <c r="O27" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.0994</v>
       </c>
     </row>
     <row r="28">
@@ -11281,10 +11281,10 @@
         <v>0.9846</v>
       </c>
       <c r="N28" t="n">
-        <v>0.0482</v>
+        <v>0.0477</v>
       </c>
       <c r="O28" t="n">
-        <v>0.09950000000000001</v>
+        <v>0.0998</v>
       </c>
     </row>
     <row r="29">
@@ -11332,10 +11332,10 @@
         <v>0.9846</v>
       </c>
       <c r="N29" t="n">
-        <v>0.0475</v>
+        <v>0.0471</v>
       </c>
       <c r="O29" t="n">
-        <v>0.0998</v>
+        <v>0.1001</v>
       </c>
     </row>
     <row r="30">
@@ -11383,10 +11383,10 @@
         <v>0.9846</v>
       </c>
       <c r="N30" t="n">
-        <v>0.0491</v>
+        <v>0.0487</v>
       </c>
       <c r="O30" t="n">
-        <v>0.1023</v>
+        <v>0.1025</v>
       </c>
     </row>
     <row r="31">
@@ -11434,10 +11434,10 @@
         <v>0.9846</v>
       </c>
       <c r="N31" t="n">
-        <v>0.0484</v>
+        <v>0.048</v>
       </c>
       <c r="O31" t="n">
-        <v>0.1013</v>
+        <v>0.1015</v>
       </c>
     </row>
     <row r="32">
@@ -11485,10 +11485,10 @@
         <v>0.6359</v>
       </c>
       <c r="N32" t="n">
-        <v>0.2398</v>
+        <v>0.2392</v>
       </c>
       <c r="O32" t="n">
-        <v>0.3064</v>
+        <v>0.3061</v>
       </c>
     </row>
     <row r="33">
@@ -11536,10 +11536,10 @@
         <v>0.6615</v>
       </c>
       <c r="N33" t="n">
-        <v>0.2424</v>
+        <v>0.2419</v>
       </c>
       <c r="O33" t="n">
-        <v>0.306</v>
+        <v>0.3057</v>
       </c>
     </row>
     <row r="34">
@@ -11587,10 +11587,10 @@
         <v>0.7026</v>
       </c>
       <c r="N34" t="n">
-        <v>0.2394</v>
+        <v>0.2389</v>
       </c>
       <c r="O34" t="n">
-        <v>0.3045</v>
+        <v>0.3041</v>
       </c>
     </row>
     <row r="35">
@@ -11638,10 +11638,10 @@
         <v>0.6768999999999999</v>
       </c>
       <c r="N35" t="n">
-        <v>0.2432</v>
+        <v>0.2429</v>
       </c>
       <c r="O35" t="n">
-        <v>0.3081</v>
+        <v>0.3079</v>
       </c>
     </row>
     <row r="36">
@@ -11689,10 +11689,10 @@
         <v>0.6462</v>
       </c>
       <c r="N36" t="n">
-        <v>0.2428</v>
+        <v>0.2424</v>
       </c>
       <c r="O36" t="n">
-        <v>0.308</v>
+        <v>0.3076</v>
       </c>
     </row>
     <row r="37">
@@ -11728,22 +11728,22 @@
         <v>195</v>
       </c>
       <c r="J37" t="n">
-        <v>0.2615</v>
+        <v>0.2581</v>
       </c>
       <c r="K37" t="n">
-        <v>0.2821</v>
+        <v>0.2795</v>
       </c>
       <c r="L37" t="n">
-        <v>0.4564</v>
+        <v>0.441</v>
       </c>
       <c r="M37" t="n">
-        <v>0.7846</v>
+        <v>0.7795</v>
       </c>
       <c r="N37" t="n">
-        <v>0.1705</v>
+        <v>0.171</v>
       </c>
       <c r="O37" t="n">
-        <v>0.2443</v>
+        <v>0.2445</v>
       </c>
     </row>
     <row r="38">
@@ -11779,22 +11779,22 @@
         <v>195</v>
       </c>
       <c r="J38" t="n">
-        <v>0.2513</v>
+        <v>0.2786</v>
       </c>
       <c r="K38" t="n">
-        <v>0.2615</v>
+        <v>0.2897</v>
       </c>
       <c r="L38" t="n">
-        <v>0.4564</v>
+        <v>0.4821</v>
       </c>
       <c r="M38" t="n">
-        <v>0.7641</v>
+        <v>0.7538</v>
       </c>
       <c r="N38" t="n">
-        <v>0.1709</v>
+        <v>0.1693</v>
       </c>
       <c r="O38" t="n">
-        <v>0.2472</v>
+        <v>0.2435</v>
       </c>
     </row>
     <row r="39">
@@ -11833,19 +11833,19 @@
         <v>0.2581</v>
       </c>
       <c r="K39" t="n">
-        <v>0.2769</v>
+        <v>0.2718</v>
       </c>
       <c r="L39" t="n">
-        <v>0.5026</v>
+        <v>0.4923</v>
       </c>
       <c r="M39" t="n">
-        <v>0.7692</v>
+        <v>0.7641</v>
       </c>
       <c r="N39" t="n">
-        <v>0.1648</v>
+        <v>0.1665</v>
       </c>
       <c r="O39" t="n">
-        <v>0.2365</v>
+        <v>0.2373</v>
       </c>
     </row>
     <row r="40">
@@ -11881,22 +11881,22 @@
         <v>195</v>
       </c>
       <c r="J40" t="n">
-        <v>0.2376</v>
+        <v>0.2308</v>
       </c>
       <c r="K40" t="n">
-        <v>0.2615</v>
+        <v>0.2564</v>
       </c>
       <c r="L40" t="n">
         <v>0.4667</v>
       </c>
       <c r="M40" t="n">
-        <v>0.7333</v>
+        <v>0.7282</v>
       </c>
       <c r="N40" t="n">
-        <v>0.1709</v>
+        <v>0.1712</v>
       </c>
       <c r="O40" t="n">
-        <v>0.2458</v>
+        <v>0.2448</v>
       </c>
     </row>
     <row r="41">
@@ -11932,22 +11932,22 @@
         <v>195</v>
       </c>
       <c r="J41" t="n">
-        <v>0.3436</v>
+        <v>0.3368</v>
       </c>
       <c r="K41" t="n">
-        <v>0.3667</v>
+        <v>0.3564</v>
       </c>
       <c r="L41" t="n">
-        <v>0.5179</v>
+        <v>0.4872</v>
       </c>
       <c r="M41" t="n">
-        <v>0.7949000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="N41" t="n">
-        <v>0.1673</v>
+        <v>0.1669</v>
       </c>
       <c r="O41" t="n">
-        <v>0.2414</v>
+        <v>0.2407</v>
       </c>
     </row>
     <row r="42">
@@ -11995,10 +11995,10 @@
         <v>0.9487</v>
       </c>
       <c r="N42" t="n">
-        <v>0.07829999999999999</v>
+        <v>0.0776</v>
       </c>
       <c r="O42" t="n">
-        <v>0.1405</v>
+        <v>0.1406</v>
       </c>
     </row>
     <row r="43">
@@ -12046,10 +12046,10 @@
         <v>0.9436</v>
       </c>
       <c r="N43" t="n">
-        <v>0.0809</v>
+        <v>0.0804</v>
       </c>
       <c r="O43" t="n">
-        <v>0.1453</v>
+        <v>0.1455</v>
       </c>
     </row>
     <row r="44">
@@ -12097,10 +12097,10 @@
         <v>0.9436</v>
       </c>
       <c r="N44" t="n">
-        <v>0.0795</v>
+        <v>0.07920000000000001</v>
       </c>
       <c r="O44" t="n">
-        <v>0.1467</v>
+        <v>0.1469</v>
       </c>
     </row>
     <row r="45">
@@ -12136,19 +12136,19 @@
         <v>195</v>
       </c>
       <c r="J45" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.8154</v>
       </c>
       <c r="K45" t="n">
-        <v>0.8333</v>
+        <v>0.8359</v>
       </c>
       <c r="L45" t="n">
-        <v>0.841</v>
+        <v>0.8462</v>
       </c>
       <c r="M45" t="n">
         <v>0.9692</v>
       </c>
       <c r="N45" t="n">
-        <v>0.0717</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="O45" t="n">
         <v>0.131</v>
@@ -12199,10 +12199,10 @@
         <v>0.9487</v>
       </c>
       <c r="N46" t="n">
-        <v>0.0781</v>
+        <v>0.0776</v>
       </c>
       <c r="O46" t="n">
-        <v>0.1391</v>
+        <v>0.1393</v>
       </c>
     </row>
     <row r="47">
@@ -12250,10 +12250,10 @@
         <v>0.6923</v>
       </c>
       <c r="N47" t="n">
-        <v>0.2373</v>
+        <v>0.2375</v>
       </c>
       <c r="O47" t="n">
-        <v>0.2983</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="48">
@@ -12301,10 +12301,10 @@
         <v>0.6923</v>
       </c>
       <c r="N48" t="n">
-        <v>0.2354</v>
+        <v>0.2352</v>
       </c>
       <c r="O48" t="n">
-        <v>0.295</v>
+        <v>0.2945</v>
       </c>
     </row>
     <row r="49">
@@ -12355,7 +12355,7 @@
         <v>0.2349</v>
       </c>
       <c r="O49" t="n">
-        <v>0.2941</v>
+        <v>0.2937</v>
       </c>
     </row>
     <row r="50">
@@ -12403,10 +12403,10 @@
         <v>0.6462</v>
       </c>
       <c r="N50" t="n">
-        <v>0.2351</v>
+        <v>0.2348</v>
       </c>
       <c r="O50" t="n">
-        <v>0.2948</v>
+        <v>0.2942</v>
       </c>
     </row>
     <row r="51">
@@ -12454,10 +12454,10 @@
         <v>0.6564</v>
       </c>
       <c r="N51" t="n">
-        <v>0.2324</v>
+        <v>0.2322</v>
       </c>
       <c r="O51" t="n">
-        <v>0.2941</v>
+        <v>0.2938</v>
       </c>
     </row>
     <row r="52">
@@ -12493,22 +12493,22 @@
         <v>195</v>
       </c>
       <c r="J52" t="n">
-        <v>0.1624</v>
+        <v>0.2205</v>
       </c>
       <c r="K52" t="n">
-        <v>0.1769</v>
+        <v>0.2308</v>
       </c>
       <c r="L52" t="n">
-        <v>0.4462</v>
+        <v>0.4615</v>
       </c>
       <c r="M52" t="n">
-        <v>0.7282</v>
+        <v>0.7641</v>
       </c>
       <c r="N52" t="n">
-        <v>0.1945</v>
+        <v>0.1953</v>
       </c>
       <c r="O52" t="n">
-        <v>0.2637</v>
+        <v>0.2631</v>
       </c>
     </row>
     <row r="53">
@@ -12544,22 +12544,22 @@
         <v>195</v>
       </c>
       <c r="J53" t="n">
-        <v>0.1966</v>
+        <v>0.2137</v>
       </c>
       <c r="K53" t="n">
-        <v>0.2026</v>
+        <v>0.2308</v>
       </c>
       <c r="L53" t="n">
-        <v>0.441</v>
+        <v>0.4513</v>
       </c>
       <c r="M53" t="n">
-        <v>0.7795</v>
+        <v>0.8</v>
       </c>
       <c r="N53" t="n">
-        <v>0.1962</v>
+        <v>0.1974</v>
       </c>
       <c r="O53" t="n">
-        <v>0.2639</v>
+        <v>0.2646</v>
       </c>
     </row>
     <row r="54">
@@ -12595,22 +12595,22 @@
         <v>195</v>
       </c>
       <c r="J54" t="n">
-        <v>0.2239</v>
+        <v>0.2205</v>
       </c>
       <c r="K54" t="n">
-        <v>0.2436</v>
+        <v>0.2385</v>
       </c>
       <c r="L54" t="n">
-        <v>0.5077</v>
+        <v>0.4821</v>
       </c>
       <c r="M54" t="n">
-        <v>0.759</v>
+        <v>0.7744</v>
       </c>
       <c r="N54" t="n">
-        <v>0.1856</v>
+        <v>0.1893</v>
       </c>
       <c r="O54" t="n">
-        <v>0.2508</v>
+        <v>0.2547</v>
       </c>
     </row>
     <row r="55">
@@ -12652,16 +12652,16 @@
         <v>0.2692</v>
       </c>
       <c r="L55" t="n">
-        <v>0.4718</v>
+        <v>0.4821</v>
       </c>
       <c r="M55" t="n">
-        <v>0.8051</v>
+        <v>0.8205</v>
       </c>
       <c r="N55" t="n">
-        <v>0.1914</v>
+        <v>0.1948</v>
       </c>
       <c r="O55" t="n">
-        <v>0.2599</v>
+        <v>0.2636</v>
       </c>
     </row>
     <row r="56">
@@ -12697,22 +12697,22 @@
         <v>195</v>
       </c>
       <c r="J56" t="n">
-        <v>0.2103</v>
+        <v>0.1453</v>
       </c>
       <c r="K56" t="n">
-        <v>0.2179</v>
+        <v>0.1513</v>
       </c>
       <c r="L56" t="n">
-        <v>0.4821</v>
+        <v>0.4513</v>
       </c>
       <c r="M56" t="n">
-        <v>0.7692</v>
+        <v>0.7436</v>
       </c>
       <c r="N56" t="n">
-        <v>0.1889</v>
+        <v>0.1909</v>
       </c>
       <c r="O56" t="n">
-        <v>0.2557</v>
+        <v>0.2568</v>
       </c>
     </row>
     <row r="57">
@@ -12760,10 +12760,10 @@
         <v>0.9641</v>
       </c>
       <c r="N57" t="n">
-        <v>0.0746</v>
+        <v>0.0741</v>
       </c>
       <c r="O57" t="n">
-        <v>0.1673</v>
+        <v>0.1674</v>
       </c>
     </row>
     <row r="58">
@@ -12811,10 +12811,10 @@
         <v>0.9692</v>
       </c>
       <c r="N58" t="n">
-        <v>0.0696</v>
+        <v>0.0692</v>
       </c>
       <c r="O58" t="n">
-        <v>0.1568</v>
+        <v>0.157</v>
       </c>
     </row>
     <row r="59">
@@ -12862,10 +12862,10 @@
         <v>0.959</v>
       </c>
       <c r="N59" t="n">
-        <v>0.0735</v>
+        <v>0.0731</v>
       </c>
       <c r="O59" t="n">
-        <v>0.1632</v>
+        <v>0.1633</v>
       </c>
     </row>
     <row r="60">
@@ -12913,10 +12913,10 @@
         <v>0.9795</v>
       </c>
       <c r="N60" t="n">
-        <v>0.074</v>
+        <v>0.0736</v>
       </c>
       <c r="O60" t="n">
-        <v>0.1667</v>
+        <v>0.1668</v>
       </c>
     </row>
     <row r="61">
@@ -12964,10 +12964,10 @@
         <v>0.9692</v>
       </c>
       <c r="N61" t="n">
-        <v>0.0711</v>
+        <v>0.0706</v>
       </c>
       <c r="O61" t="n">
-        <v>0.1572</v>
+        <v>0.1574</v>
       </c>
     </row>
     <row r="62">
@@ -13013,10 +13013,10 @@
         <v>0.7513</v>
       </c>
       <c r="N62" t="n">
-        <v>0.232</v>
+        <v>0.2319</v>
       </c>
       <c r="O62" t="n">
-        <v>0.3017</v>
+        <v>0.3016</v>
       </c>
     </row>
     <row r="63">
@@ -13062,7 +13062,7 @@
         <v>0.7268</v>
       </c>
       <c r="N63" t="n">
-        <v>0.2293</v>
+        <v>0.2294</v>
       </c>
       <c r="O63" t="n">
         <v>0.3008</v>
@@ -13111,7 +13111,7 @@
         <v>0.7083</v>
       </c>
       <c r="N64" t="n">
-        <v>0.2355</v>
+        <v>0.2356</v>
       </c>
       <c r="O64" t="n">
         <v>0.307</v>
@@ -13160,10 +13160,10 @@
         <v>0.7113</v>
       </c>
       <c r="N65" t="n">
-        <v>0.2313</v>
+        <v>0.231</v>
       </c>
       <c r="O65" t="n">
-        <v>0.299</v>
+        <v>0.2987</v>
       </c>
     </row>
     <row r="66">
@@ -13209,10 +13209,10 @@
         <v>0.7128</v>
       </c>
       <c r="N66" t="n">
-        <v>0.2296</v>
+        <v>0.2292</v>
       </c>
       <c r="O66" t="n">
-        <v>0.301</v>
+        <v>0.3006</v>
       </c>
     </row>
     <row r="67">
@@ -13246,19 +13246,19 @@
         <v>195</v>
       </c>
       <c r="J67" t="n">
-        <v>0.3299</v>
+        <v>0.3436</v>
       </c>
       <c r="K67" t="n">
-        <v>0.3564</v>
+        <v>0.3615</v>
       </c>
       <c r="L67" t="n">
-        <v>0.5692</v>
+        <v>0.5744</v>
       </c>
       <c r="M67" t="n">
-        <v>0.7949000000000001</v>
+        <v>0.8051</v>
       </c>
       <c r="N67" t="n">
-        <v>0.1675</v>
+        <v>0.1682</v>
       </c>
       <c r="O67" t="n">
         <v>0.2376</v>
@@ -13295,22 +13295,22 @@
         <v>195</v>
       </c>
       <c r="J68" t="n">
-        <v>0.3162</v>
+        <v>0.3368</v>
       </c>
       <c r="K68" t="n">
-        <v>0.3462</v>
+        <v>0.3667</v>
       </c>
       <c r="L68" t="n">
-        <v>0.5436</v>
+        <v>0.5641</v>
       </c>
       <c r="M68" t="n">
-        <v>0.8359</v>
+        <v>0.8462</v>
       </c>
       <c r="N68" t="n">
-        <v>0.1655</v>
+        <v>0.1667</v>
       </c>
       <c r="O68" t="n">
-        <v>0.2347</v>
+        <v>0.2346</v>
       </c>
     </row>
     <row r="69">
@@ -13344,22 +13344,22 @@
         <v>195</v>
       </c>
       <c r="J69" t="n">
-        <v>0.2855</v>
+        <v>0.2581</v>
       </c>
       <c r="K69" t="n">
-        <v>0.3128</v>
+        <v>0.2821</v>
       </c>
       <c r="L69" t="n">
-        <v>0.5077</v>
+        <v>0.4974</v>
       </c>
       <c r="M69" t="n">
         <v>0.8103</v>
       </c>
       <c r="N69" t="n">
-        <v>0.1675</v>
+        <v>0.168</v>
       </c>
       <c r="O69" t="n">
-        <v>0.2364</v>
+        <v>0.2366</v>
       </c>
     </row>
     <row r="70">
@@ -13393,22 +13393,22 @@
         <v>195</v>
       </c>
       <c r="J70" t="n">
-        <v>0.3573</v>
+        <v>0.2855</v>
       </c>
       <c r="K70" t="n">
-        <v>0.3769</v>
+        <v>0.3026</v>
       </c>
       <c r="L70" t="n">
-        <v>0.5487</v>
+        <v>0.5282</v>
       </c>
       <c r="M70" t="n">
-        <v>0.8154</v>
+        <v>0.7795</v>
       </c>
       <c r="N70" t="n">
-        <v>0.1638</v>
+        <v>0.1674</v>
       </c>
       <c r="O70" t="n">
-        <v>0.233</v>
+        <v>0.2374</v>
       </c>
     </row>
     <row r="71">
@@ -13442,22 +13442,22 @@
         <v>195</v>
       </c>
       <c r="J71" t="n">
-        <v>0.3504</v>
+        <v>0.3094</v>
       </c>
       <c r="K71" t="n">
-        <v>0.3769</v>
+        <v>0.341</v>
       </c>
       <c r="L71" t="n">
-        <v>0.5538</v>
+        <v>0.5128</v>
       </c>
       <c r="M71" t="n">
-        <v>0.8205</v>
+        <v>0.8154</v>
       </c>
       <c r="N71" t="n">
-        <v>0.1691</v>
+        <v>0.1683</v>
       </c>
       <c r="O71" t="n">
-        <v>0.237</v>
+        <v>0.2364</v>
       </c>
     </row>
     <row r="72">
@@ -13503,10 +13503,10 @@
         <v>0.9846</v>
       </c>
       <c r="N72" t="n">
-        <v>0.0399</v>
+        <v>0.0395</v>
       </c>
       <c r="O72" t="n">
-        <v>0.07770000000000001</v>
+        <v>0.0781</v>
       </c>
     </row>
     <row r="73">
@@ -13540,22 +13540,22 @@
         <v>195</v>
       </c>
       <c r="J73" t="n">
-        <v>0.8935</v>
+        <v>0.89</v>
       </c>
       <c r="K73" t="n">
-        <v>0.9072</v>
+        <v>0.9046</v>
       </c>
       <c r="L73" t="n">
-        <v>0.9021</v>
+        <v>0.8969</v>
       </c>
       <c r="M73" t="n">
         <v>0.9742</v>
       </c>
       <c r="N73" t="n">
-        <v>0.0484</v>
+        <v>0.0465</v>
       </c>
       <c r="O73" t="n">
-        <v>0.0963</v>
+        <v>0.09569999999999999</v>
       </c>
     </row>
     <row r="74">
@@ -13601,10 +13601,10 @@
         <v>0.9744</v>
       </c>
       <c r="N74" t="n">
-        <v>0.0486</v>
+        <v>0.0462</v>
       </c>
       <c r="O74" t="n">
-        <v>0.0954</v>
+        <v>0.09429999999999999</v>
       </c>
     </row>
     <row r="75">
@@ -13650,10 +13650,10 @@
         <v>0.9795</v>
       </c>
       <c r="N75" t="n">
-        <v>0.0452</v>
+        <v>0.0427</v>
       </c>
       <c r="O75" t="n">
-        <v>0.0854</v>
+        <v>0.0839</v>
       </c>
     </row>
     <row r="76">
@@ -13687,22 +13687,22 @@
         <v>195</v>
       </c>
       <c r="J76" t="n">
-        <v>0.894</v>
+        <v>0.8974</v>
       </c>
       <c r="K76" t="n">
+        <v>0.9103</v>
+      </c>
+      <c r="L76" t="n">
         <v>0.9077</v>
-      </c>
-      <c r="L76" t="n">
-        <v>0.9026</v>
       </c>
       <c r="M76" t="n">
         <v>0.9744</v>
       </c>
       <c r="N76" t="n">
-        <v>0.0517</v>
+        <v>0.0493</v>
       </c>
       <c r="O76" t="n">
-        <v>0.1075</v>
+        <v>0.1066</v>
       </c>
     </row>
     <row r="77">
@@ -13748,10 +13748,10 @@
         <v>0.7026</v>
       </c>
       <c r="N77" t="n">
-        <v>0.2171</v>
+        <v>0.2164</v>
       </c>
       <c r="O77" t="n">
-        <v>0.2929</v>
+        <v>0.2922</v>
       </c>
     </row>
     <row r="78">
@@ -13797,10 +13797,10 @@
         <v>0.6718</v>
       </c>
       <c r="N78" t="n">
-        <v>0.2193</v>
+        <v>0.2188</v>
       </c>
       <c r="O78" t="n">
-        <v>0.2966</v>
+        <v>0.296</v>
       </c>
     </row>
     <row r="79">
@@ -13846,10 +13846,10 @@
         <v>0.7077</v>
       </c>
       <c r="N79" t="n">
-        <v>0.2203</v>
+        <v>0.2198</v>
       </c>
       <c r="O79" t="n">
-        <v>0.2968</v>
+        <v>0.2961</v>
       </c>
     </row>
     <row r="80">
@@ -13895,10 +13895,10 @@
         <v>0.6923</v>
       </c>
       <c r="N80" t="n">
-        <v>0.2215</v>
+        <v>0.2209</v>
       </c>
       <c r="O80" t="n">
-        <v>0.2976</v>
+        <v>0.297</v>
       </c>
     </row>
     <row r="81">
@@ -13944,10 +13944,10 @@
         <v>0.7128</v>
       </c>
       <c r="N81" t="n">
-        <v>0.2197</v>
+        <v>0.2191</v>
       </c>
       <c r="O81" t="n">
-        <v>0.296</v>
+        <v>0.2954</v>
       </c>
     </row>
     <row r="82">
@@ -13970,33 +13970,33 @@
         <v>1</v>
       </c>
       <c r="E82" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I82" t="n">
         <v>195</v>
       </c>
       <c r="J82" t="n">
-        <v>0.2815</v>
+        <v>0.2852</v>
       </c>
       <c r="K82" t="n">
-        <v>0.2979</v>
+        <v>0.3041</v>
       </c>
       <c r="L82" t="n">
-        <v>0.456</v>
+        <v>0.4691</v>
       </c>
       <c r="M82" t="n">
-        <v>0.8031</v>
+        <v>0.8041</v>
       </c>
       <c r="N82" t="n">
-        <v>0.1588</v>
+        <v>0.1587</v>
       </c>
       <c r="O82" t="n">
-        <v>0.2339</v>
+        <v>0.2327</v>
       </c>
     </row>
     <row r="83">
@@ -14030,22 +14030,22 @@
         <v>195</v>
       </c>
       <c r="J83" t="n">
-        <v>0.3333</v>
+        <v>0.3299</v>
       </c>
       <c r="K83" t="n">
         <v>0.3523</v>
       </c>
       <c r="L83" t="n">
-        <v>0.5078</v>
+        <v>0.513</v>
       </c>
       <c r="M83" t="n">
         <v>0.7927</v>
       </c>
       <c r="N83" t="n">
-        <v>0.1573</v>
+        <v>0.1575</v>
       </c>
       <c r="O83" t="n">
-        <v>0.2313</v>
+        <v>0.2307</v>
       </c>
     </row>
     <row r="84">
@@ -14068,33 +14068,33 @@
         <v>3</v>
       </c>
       <c r="E84" t="n">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I84" t="n">
         <v>195</v>
       </c>
       <c r="J84" t="n">
-        <v>0.3019</v>
+        <v>0.2953</v>
       </c>
       <c r="K84" t="n">
-        <v>0.3194</v>
+        <v>0.3161</v>
       </c>
       <c r="L84" t="n">
-        <v>0.4712</v>
+        <v>0.4663</v>
       </c>
       <c r="M84" t="n">
-        <v>0.7906</v>
+        <v>0.7927</v>
       </c>
       <c r="N84" t="n">
-        <v>0.1585</v>
+        <v>0.1586</v>
       </c>
       <c r="O84" t="n">
-        <v>0.2325</v>
+        <v>0.2312</v>
       </c>
     </row>
     <row r="85">
@@ -14117,33 +14117,33 @@
         <v>4</v>
       </c>
       <c r="E85" t="n">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I85" t="n">
         <v>195</v>
       </c>
       <c r="J85" t="n">
-        <v>0.3014</v>
+        <v>0.3195</v>
       </c>
       <c r="K85" t="n">
-        <v>0.3112</v>
+        <v>0.3316</v>
       </c>
       <c r="L85" t="n">
-        <v>0.4628</v>
+        <v>0.487</v>
       </c>
       <c r="M85" t="n">
-        <v>0.7872</v>
+        <v>0.7927</v>
       </c>
       <c r="N85" t="n">
-        <v>0.1595</v>
+        <v>0.1572</v>
       </c>
       <c r="O85" t="n">
-        <v>0.2317</v>
+        <v>0.2283</v>
       </c>
     </row>
     <row r="86">
@@ -14166,33 +14166,33 @@
         <v>5</v>
       </c>
       <c r="E86" t="n">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I86" t="n">
         <v>195</v>
       </c>
       <c r="J86" t="n">
-        <v>0.3053</v>
+        <v>0.3194</v>
       </c>
       <c r="K86" t="n">
-        <v>0.3211</v>
+        <v>0.3359</v>
       </c>
       <c r="L86" t="n">
-        <v>0.4632</v>
+        <v>0.5</v>
       </c>
       <c r="M86" t="n">
-        <v>0.7947</v>
+        <v>0.7969000000000001</v>
       </c>
       <c r="N86" t="n">
         <v>0.1599</v>
       </c>
       <c r="O86" t="n">
-        <v>0.2343</v>
+        <v>0.2328</v>
       </c>
     </row>
     <row r="87">
@@ -14238,10 +14238,10 @@
         <v>0.9846</v>
       </c>
       <c r="N87" t="n">
-        <v>0.0474</v>
+        <v>0.0469</v>
       </c>
       <c r="O87" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.0994</v>
       </c>
     </row>
     <row r="88">
@@ -14287,10 +14287,10 @@
         <v>0.9846</v>
       </c>
       <c r="N88" t="n">
-        <v>0.0482</v>
+        <v>0.0477</v>
       </c>
       <c r="O88" t="n">
-        <v>0.09950000000000001</v>
+        <v>0.0998</v>
       </c>
     </row>
     <row r="89">
@@ -14336,10 +14336,10 @@
         <v>0.9846</v>
       </c>
       <c r="N89" t="n">
-        <v>0.0475</v>
+        <v>0.0471</v>
       </c>
       <c r="O89" t="n">
-        <v>0.0998</v>
+        <v>0.1001</v>
       </c>
     </row>
     <row r="90">
@@ -14385,10 +14385,10 @@
         <v>0.9846</v>
       </c>
       <c r="N90" t="n">
-        <v>0.0491</v>
+        <v>0.0487</v>
       </c>
       <c r="O90" t="n">
-        <v>0.1023</v>
+        <v>0.1025</v>
       </c>
     </row>
     <row r="91">
@@ -14434,10 +14434,10 @@
         <v>0.9846</v>
       </c>
       <c r="N91" t="n">
-        <v>0.0484</v>
+        <v>0.048</v>
       </c>
       <c r="O91" t="n">
-        <v>0.1013</v>
+        <v>0.1015</v>
       </c>
     </row>
     <row r="92">
@@ -14483,10 +14483,10 @@
         <v>0.6359</v>
       </c>
       <c r="N92" t="n">
-        <v>0.2398</v>
+        <v>0.2392</v>
       </c>
       <c r="O92" t="n">
-        <v>0.3064</v>
+        <v>0.3061</v>
       </c>
     </row>
     <row r="93">
@@ -14532,10 +14532,10 @@
         <v>0.6615</v>
       </c>
       <c r="N93" t="n">
-        <v>0.2424</v>
+        <v>0.2419</v>
       </c>
       <c r="O93" t="n">
-        <v>0.306</v>
+        <v>0.3057</v>
       </c>
     </row>
     <row r="94">
@@ -14581,10 +14581,10 @@
         <v>0.7026</v>
       </c>
       <c r="N94" t="n">
-        <v>0.2394</v>
+        <v>0.2389</v>
       </c>
       <c r="O94" t="n">
-        <v>0.3045</v>
+        <v>0.3041</v>
       </c>
     </row>
     <row r="95">
@@ -14630,10 +14630,10 @@
         <v>0.6768999999999999</v>
       </c>
       <c r="N95" t="n">
-        <v>0.2432</v>
+        <v>0.2429</v>
       </c>
       <c r="O95" t="n">
-        <v>0.3081</v>
+        <v>0.3079</v>
       </c>
     </row>
     <row r="96">
@@ -14679,10 +14679,10 @@
         <v>0.6462</v>
       </c>
       <c r="N96" t="n">
-        <v>0.2428</v>
+        <v>0.2424</v>
       </c>
       <c r="O96" t="n">
-        <v>0.308</v>
+        <v>0.3076</v>
       </c>
     </row>
     <row r="97">
@@ -14716,22 +14716,22 @@
         <v>195</v>
       </c>
       <c r="J97" t="n">
-        <v>0.2615</v>
+        <v>0.2581</v>
       </c>
       <c r="K97" t="n">
-        <v>0.2821</v>
+        <v>0.2795</v>
       </c>
       <c r="L97" t="n">
-        <v>0.4564</v>
+        <v>0.441</v>
       </c>
       <c r="M97" t="n">
-        <v>0.7846</v>
+        <v>0.7795</v>
       </c>
       <c r="N97" t="n">
-        <v>0.1705</v>
+        <v>0.171</v>
       </c>
       <c r="O97" t="n">
-        <v>0.2443</v>
+        <v>0.2445</v>
       </c>
     </row>
     <row r="98">
@@ -14765,22 +14765,22 @@
         <v>195</v>
       </c>
       <c r="J98" t="n">
-        <v>0.2513</v>
+        <v>0.2786</v>
       </c>
       <c r="K98" t="n">
-        <v>0.2615</v>
+        <v>0.2897</v>
       </c>
       <c r="L98" t="n">
-        <v>0.4564</v>
+        <v>0.4821</v>
       </c>
       <c r="M98" t="n">
-        <v>0.7641</v>
+        <v>0.7538</v>
       </c>
       <c r="N98" t="n">
-        <v>0.1709</v>
+        <v>0.1693</v>
       </c>
       <c r="O98" t="n">
-        <v>0.2472</v>
+        <v>0.2435</v>
       </c>
     </row>
     <row r="99">
@@ -14817,19 +14817,19 @@
         <v>0.2581</v>
       </c>
       <c r="K99" t="n">
-        <v>0.2769</v>
+        <v>0.2718</v>
       </c>
       <c r="L99" t="n">
-        <v>0.5026</v>
+        <v>0.4923</v>
       </c>
       <c r="M99" t="n">
-        <v>0.7692</v>
+        <v>0.7641</v>
       </c>
       <c r="N99" t="n">
-        <v>0.1648</v>
+        <v>0.1665</v>
       </c>
       <c r="O99" t="n">
-        <v>0.2365</v>
+        <v>0.2373</v>
       </c>
     </row>
     <row r="100">
@@ -14863,22 +14863,22 @@
         <v>195</v>
       </c>
       <c r="J100" t="n">
-        <v>0.2376</v>
+        <v>0.2308</v>
       </c>
       <c r="K100" t="n">
-        <v>0.2615</v>
+        <v>0.2564</v>
       </c>
       <c r="L100" t="n">
         <v>0.4667</v>
       </c>
       <c r="M100" t="n">
-        <v>0.7333</v>
+        <v>0.7282</v>
       </c>
       <c r="N100" t="n">
-        <v>0.1709</v>
+        <v>0.1712</v>
       </c>
       <c r="O100" t="n">
-        <v>0.2458</v>
+        <v>0.2448</v>
       </c>
     </row>
     <row r="101">
@@ -14912,22 +14912,22 @@
         <v>195</v>
       </c>
       <c r="J101" t="n">
-        <v>0.3436</v>
+        <v>0.3368</v>
       </c>
       <c r="K101" t="n">
-        <v>0.3667</v>
+        <v>0.3564</v>
       </c>
       <c r="L101" t="n">
-        <v>0.5179</v>
+        <v>0.4872</v>
       </c>
       <c r="M101" t="n">
-        <v>0.7949000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="N101" t="n">
-        <v>0.1673</v>
+        <v>0.1669</v>
       </c>
       <c r="O101" t="n">
-        <v>0.2414</v>
+        <v>0.2407</v>
       </c>
     </row>
     <row r="102">
@@ -14973,10 +14973,10 @@
         <v>0.9706</v>
       </c>
       <c r="N102" t="n">
-        <v>0.0516</v>
+        <v>0.0509</v>
       </c>
       <c r="O102" t="n">
-        <v>0.09950000000000001</v>
+        <v>0.09959999999999999</v>
       </c>
     </row>
     <row r="103">
@@ -15022,10 +15022,10 @@
         <v>0.9762999999999999</v>
       </c>
       <c r="N103" t="n">
-        <v>0.052</v>
+        <v>0.0514</v>
       </c>
       <c r="O103" t="n">
-        <v>0.1014</v>
+        <v>0.1016</v>
       </c>
     </row>
     <row r="104">
@@ -15071,10 +15071,10 @@
         <v>0.9828</v>
       </c>
       <c r="N104" t="n">
-        <v>0.0548</v>
+        <v>0.0545</v>
       </c>
       <c r="O104" t="n">
-        <v>0.1086</v>
+        <v>0.1089</v>
       </c>
     </row>
     <row r="105">
@@ -15108,19 +15108,19 @@
         <v>195</v>
       </c>
       <c r="J105" t="n">
-        <v>0.8971</v>
+        <v>0.901</v>
       </c>
       <c r="K105" t="n">
-        <v>0.9171</v>
+        <v>0.92</v>
       </c>
       <c r="L105" t="n">
-        <v>0.9086</v>
+        <v>0.9143</v>
       </c>
       <c r="M105" t="n">
         <v>0.9943</v>
       </c>
       <c r="N105" t="n">
-        <v>0.0518</v>
+        <v>0.051</v>
       </c>
       <c r="O105" t="n">
         <v>0.0989</v>
@@ -15169,10 +15169,10 @@
         <v>0.9824000000000001</v>
       </c>
       <c r="N106" t="n">
-        <v>0.0522</v>
+        <v>0.0516</v>
       </c>
       <c r="O106" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.0984</v>
       </c>
     </row>
     <row r="107">
@@ -15218,10 +15218,10 @@
         <v>0.6923</v>
       </c>
       <c r="N107" t="n">
-        <v>0.2373</v>
+        <v>0.2375</v>
       </c>
       <c r="O107" t="n">
-        <v>0.2983</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="108">
@@ -15267,10 +15267,10 @@
         <v>0.6923</v>
       </c>
       <c r="N108" t="n">
-        <v>0.2354</v>
+        <v>0.2352</v>
       </c>
       <c r="O108" t="n">
-        <v>0.295</v>
+        <v>0.2945</v>
       </c>
     </row>
     <row r="109">
@@ -15316,10 +15316,10 @@
         <v>0.701</v>
       </c>
       <c r="N109" t="n">
-        <v>0.2343</v>
+        <v>0.2342</v>
       </c>
       <c r="O109" t="n">
-        <v>0.2934</v>
+        <v>0.293</v>
       </c>
     </row>
     <row r="110">
@@ -15365,10 +15365,10 @@
         <v>0.6462</v>
       </c>
       <c r="N110" t="n">
-        <v>0.2351</v>
+        <v>0.2348</v>
       </c>
       <c r="O110" t="n">
-        <v>0.2948</v>
+        <v>0.2942</v>
       </c>
     </row>
     <row r="111">
@@ -15414,10 +15414,10 @@
         <v>0.6546</v>
       </c>
       <c r="N111" t="n">
-        <v>0.2327</v>
+        <v>0.2326</v>
       </c>
       <c r="O111" t="n">
-        <v>0.2946</v>
+        <v>0.2943</v>
       </c>
     </row>
     <row r="112">
@@ -15451,22 +15451,22 @@
         <v>195</v>
       </c>
       <c r="J112" t="n">
-        <v>0.1624</v>
+        <v>0.2205</v>
       </c>
       <c r="K112" t="n">
-        <v>0.1769</v>
+        <v>0.2308</v>
       </c>
       <c r="L112" t="n">
-        <v>0.4462</v>
+        <v>0.4615</v>
       </c>
       <c r="M112" t="n">
-        <v>0.7282</v>
+        <v>0.7641</v>
       </c>
       <c r="N112" t="n">
-        <v>0.1945</v>
+        <v>0.1953</v>
       </c>
       <c r="O112" t="n">
-        <v>0.2637</v>
+        <v>0.2631</v>
       </c>
     </row>
     <row r="113">
@@ -15500,22 +15500,22 @@
         <v>195</v>
       </c>
       <c r="J113" t="n">
-        <v>0.1966</v>
+        <v>0.2137</v>
       </c>
       <c r="K113" t="n">
-        <v>0.2026</v>
+        <v>0.2308</v>
       </c>
       <c r="L113" t="n">
-        <v>0.441</v>
+        <v>0.4513</v>
       </c>
       <c r="M113" t="n">
-        <v>0.7795</v>
+        <v>0.8</v>
       </c>
       <c r="N113" t="n">
-        <v>0.1962</v>
+        <v>0.1974</v>
       </c>
       <c r="O113" t="n">
-        <v>0.2639</v>
+        <v>0.2646</v>
       </c>
     </row>
     <row r="114">
@@ -15549,22 +15549,22 @@
         <v>195</v>
       </c>
       <c r="J114" t="n">
-        <v>0.2239</v>
+        <v>0.2205</v>
       </c>
       <c r="K114" t="n">
-        <v>0.2436</v>
+        <v>0.2385</v>
       </c>
       <c r="L114" t="n">
-        <v>0.5077</v>
+        <v>0.4821</v>
       </c>
       <c r="M114" t="n">
-        <v>0.759</v>
+        <v>0.7744</v>
       </c>
       <c r="N114" t="n">
-        <v>0.1856</v>
+        <v>0.1893</v>
       </c>
       <c r="O114" t="n">
-        <v>0.2508</v>
+        <v>0.2547</v>
       </c>
     </row>
     <row r="115">
@@ -15604,16 +15604,16 @@
         <v>0.2692</v>
       </c>
       <c r="L115" t="n">
-        <v>0.4718</v>
+        <v>0.4821</v>
       </c>
       <c r="M115" t="n">
-        <v>0.8051</v>
+        <v>0.8205</v>
       </c>
       <c r="N115" t="n">
-        <v>0.1914</v>
+        <v>0.1948</v>
       </c>
       <c r="O115" t="n">
-        <v>0.2599</v>
+        <v>0.2636</v>
       </c>
     </row>
     <row r="116">
@@ -15647,22 +15647,22 @@
         <v>195</v>
       </c>
       <c r="J116" t="n">
-        <v>0.2103</v>
+        <v>0.1453</v>
       </c>
       <c r="K116" t="n">
-        <v>0.2179</v>
+        <v>0.1513</v>
       </c>
       <c r="L116" t="n">
-        <v>0.4821</v>
+        <v>0.4513</v>
       </c>
       <c r="M116" t="n">
-        <v>0.7692</v>
+        <v>0.7436</v>
       </c>
       <c r="N116" t="n">
-        <v>0.1889</v>
+        <v>0.1909</v>
       </c>
       <c r="O116" t="n">
-        <v>0.2557</v>
+        <v>0.2568</v>
       </c>
     </row>
     <row r="117">
@@ -15708,10 +15708,10 @@
         <v>0.9691</v>
       </c>
       <c r="N117" t="n">
-        <v>0.0733</v>
+        <v>0.07290000000000001</v>
       </c>
       <c r="O117" t="n">
-        <v>0.1659</v>
+        <v>0.1661</v>
       </c>
     </row>
     <row r="118">
@@ -15757,10 +15757,10 @@
         <v>0.9692</v>
       </c>
       <c r="N118" t="n">
-        <v>0.0696</v>
+        <v>0.0692</v>
       </c>
       <c r="O118" t="n">
-        <v>0.1568</v>
+        <v>0.157</v>
       </c>
     </row>
     <row r="119">
@@ -15806,10 +15806,10 @@
         <v>0.959</v>
       </c>
       <c r="N119" t="n">
-        <v>0.0735</v>
+        <v>0.0731</v>
       </c>
       <c r="O119" t="n">
-        <v>0.1632</v>
+        <v>0.1633</v>
       </c>
     </row>
     <row r="120">
@@ -15855,10 +15855,10 @@
         <v>0.9794</v>
       </c>
       <c r="N120" t="n">
-        <v>0.0736</v>
+        <v>0.0731</v>
       </c>
       <c r="O120" t="n">
-        <v>0.1665</v>
+        <v>0.1666</v>
       </c>
     </row>
     <row r="121">
@@ -15904,10 +15904,10 @@
         <v>0.9692</v>
       </c>
       <c r="N121" t="n">
-        <v>0.0711</v>
+        <v>0.0706</v>
       </c>
       <c r="O121" t="n">
-        <v>0.1572</v>
+        <v>0.1574</v>
       </c>
     </row>
   </sheetData>

</xml_diff>